<commit_message>
first round report.code breaks down, not able to replicate output
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/floswald/.julia/dev/JPEtools/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\broos.nafthali\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{957E4354-791A-4942-ABF7-9C88724FEAB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C386DC8-61C7-4B95-BB31-16F6529FD76D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="21900" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="60">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -46,13 +46,172 @@
   </si>
   <si>
     <t>In-text numbers</t>
+  </si>
+  <si>
+    <t>Figure 1</t>
+  </si>
+  <si>
+    <t>Figure 2</t>
+  </si>
+  <si>
+    <t>Figure 3</t>
+  </si>
+  <si>
+    <t>Figure 4</t>
+  </si>
+  <si>
+    <t>Figure 5</t>
+  </si>
+  <si>
+    <t>Figure 6</t>
+  </si>
+  <si>
+    <t>Table 1</t>
+  </si>
+  <si>
+    <t>Figure 0A.1</t>
+  </si>
+  <si>
+    <t>Figure 0A.2</t>
+  </si>
+  <si>
+    <t>Figure 0A.3</t>
+  </si>
+  <si>
+    <t>Figure 0A.4</t>
+  </si>
+  <si>
+    <t>Figure 0A.5</t>
+  </si>
+  <si>
+    <t>Figure 0A.6</t>
+  </si>
+  <si>
+    <t>Table 0A.1</t>
+  </si>
+  <si>
+    <t>Table 0A.2</t>
+  </si>
+  <si>
+    <t>Table 0A.3</t>
+  </si>
+  <si>
+    <t>Figure 0A.7</t>
+  </si>
+  <si>
+    <t>Figure 0A.8</t>
+  </si>
+  <si>
+    <t>Figure 0A.9</t>
+  </si>
+  <si>
+    <t>Figure 0A.10</t>
+  </si>
+  <si>
+    <t>Figure 0A.11</t>
+  </si>
+  <si>
+    <t>Figure 0A.12</t>
+  </si>
+  <si>
+    <t>Figure 0A.13</t>
+  </si>
+  <si>
+    <t>Figure 0A.14</t>
+  </si>
+  <si>
+    <t>Figure 0A.15</t>
+  </si>
+  <si>
+    <t>Figure 0A.16</t>
+  </si>
+  <si>
+    <t>Figure 0A.17</t>
+  </si>
+  <si>
+    <t>Figure 0A.18</t>
+  </si>
+  <si>
+    <t>Figure 0A.19</t>
+  </si>
+  <si>
+    <t>Figure 0A.20</t>
+  </si>
+  <si>
+    <t>Figure 0A.21</t>
+  </si>
+  <si>
+    <t>Figure 0A.22</t>
+  </si>
+  <si>
+    <t>Figure 0A.23</t>
+  </si>
+  <si>
+    <t>Figure 0A.24</t>
+  </si>
+  <si>
+    <t>Figure 0A.25</t>
+  </si>
+  <si>
+    <t>Figure 0A.26</t>
+  </si>
+  <si>
+    <t>Figure 0A.27</t>
+  </si>
+  <si>
+    <t>Figure 0A.28</t>
+  </si>
+  <si>
+    <t>Figure 0A.29</t>
+  </si>
+  <si>
+    <t>Figure 0A.30</t>
+  </si>
+  <si>
+    <t>Figure 0A.31</t>
+  </si>
+  <si>
+    <t>Figure 0A.32</t>
+  </si>
+  <si>
+    <t>Figure 0A.33</t>
+  </si>
+  <si>
+    <t>Matlab</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>p01_TRAINS_clean_data_v1_AAG.do</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>p02_eora_trade_matrix_clean.do</t>
+  </si>
+  <si>
+    <t>p02_quantiles_colombia_firmexports.do</t>
+  </si>
+  <si>
+    <t>p02_ChinaData_Morrow.do</t>
+  </si>
+  <si>
+    <t>p03_Create_Tariffs.do</t>
+  </si>
+  <si>
+    <t>p04_Sample_Creation.do</t>
+  </si>
+  <si>
+    <t>p05_Sample_Creation_HS2.do</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -64,6 +223,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -434,22 +599,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L44"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -465,42 +629,539 @@
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" t="s">
+        <v>50</v>
+      </c>
+      <c r="G10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" t="s">
+        <v>50</v>
+      </c>
+      <c r="G13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E14" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E15" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="E16" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" t="s">
+        <v>50</v>
+      </c>
+      <c r="G16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E17" t="s">
+        <v>22</v>
+      </c>
+      <c r="F17" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" t="s">
+        <v>50</v>
+      </c>
+      <c r="G18" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>24</v>
+      </c>
+      <c r="F19" t="s">
+        <v>50</v>
+      </c>
+      <c r="G19" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" t="s">
+        <v>50</v>
+      </c>
+      <c r="G20" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>26</v>
+      </c>
+      <c r="F21" t="s">
+        <v>50</v>
+      </c>
+      <c r="G21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>27</v>
+      </c>
+      <c r="F22" t="s">
+        <v>50</v>
+      </c>
+      <c r="G22" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E23" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" t="s">
+        <v>50</v>
+      </c>
+      <c r="G23" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F24" t="s">
+        <v>50</v>
+      </c>
+      <c r="G24" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E25" t="s">
+        <v>30</v>
+      </c>
+      <c r="F25" t="s">
+        <v>50</v>
+      </c>
+      <c r="G25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E26" t="s">
+        <v>31</v>
+      </c>
+      <c r="F26" t="s">
+        <v>50</v>
+      </c>
+      <c r="G26" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E27" t="s">
+        <v>32</v>
+      </c>
+      <c r="F27" t="s">
+        <v>50</v>
+      </c>
+      <c r="G27" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E28" t="s">
+        <v>33</v>
+      </c>
+      <c r="F28" t="s">
+        <v>50</v>
+      </c>
+      <c r="G28" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E29" t="s">
+        <v>34</v>
+      </c>
+      <c r="F29" t="s">
+        <v>50</v>
+      </c>
+      <c r="G29" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E30" t="s">
+        <v>35</v>
+      </c>
+      <c r="F30" t="s">
+        <v>50</v>
+      </c>
+      <c r="G30" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="31" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E31" t="s">
+        <v>36</v>
+      </c>
+      <c r="F31" t="s">
+        <v>50</v>
+      </c>
+      <c r="G31" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="32" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E32" t="s">
+        <v>37</v>
+      </c>
+      <c r="F32" t="s">
+        <v>50</v>
+      </c>
+      <c r="G32" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="33" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E33" t="s">
+        <v>38</v>
+      </c>
+      <c r="F33" t="s">
+        <v>50</v>
+      </c>
+      <c r="G33" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="34" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E34" t="s">
+        <v>39</v>
+      </c>
+      <c r="F34" t="s">
+        <v>50</v>
+      </c>
+      <c r="G34" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="35" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E35" t="s">
+        <v>40</v>
+      </c>
+      <c r="F35" t="s">
+        <v>50</v>
+      </c>
+      <c r="G35" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="36" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E36" t="s">
+        <v>41</v>
+      </c>
+      <c r="F36" t="s">
+        <v>50</v>
+      </c>
+      <c r="G36" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="37" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E37" t="s">
+        <v>42</v>
+      </c>
+      <c r="F37" t="s">
+        <v>50</v>
+      </c>
+      <c r="G37" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="38" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E38" t="s">
+        <v>43</v>
+      </c>
+      <c r="F38" t="s">
+        <v>50</v>
+      </c>
+      <c r="G38" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="39" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E39" t="s">
+        <v>44</v>
+      </c>
+      <c r="F39" t="s">
+        <v>50</v>
+      </c>
+      <c r="G39" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="40" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E40" t="s">
+        <v>45</v>
+      </c>
+      <c r="F40" t="s">
+        <v>50</v>
+      </c>
+      <c r="G40" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="41" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E41" t="s">
+        <v>46</v>
+      </c>
+      <c r="F41" t="s">
+        <v>50</v>
+      </c>
+      <c r="G41" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="42" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E42" t="s">
+        <v>47</v>
+      </c>
+      <c r="F42" t="s">
+        <v>50</v>
+      </c>
+      <c r="G42" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="43" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E43" t="s">
+        <v>48</v>
+      </c>
+      <c r="F43" t="s">
+        <v>50</v>
+      </c>
+      <c r="G43" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="44" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E44" t="s">
+        <v>49</v>
+      </c>
+      <c r="F44" t="s">
+        <v>50</v>
+      </c>
+      <c r="G44" t="s">
+        <v>51</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
round2, a few scripts broke down but majority of the output is generated
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\broos.nafthali\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C386DC8-61C7-4B95-BB31-16F6529FD76D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C114B4-C98E-42FE-AF05-F2DF5806318D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="65">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -205,6 +205,21 @@
   </si>
   <si>
     <t>p05_Sample_Creation_HS2.do</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>Table OA.4</t>
+  </si>
+  <si>
+    <t>Stata</t>
+  </si>
+  <si>
+    <t>Table OA.5</t>
+  </si>
+  <si>
+    <t>Table OA.6</t>
   </si>
 </sst>
 </file>
@@ -599,7 +614,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
@@ -659,7 +674,7 @@
         <v>50</v>
       </c>
       <c r="G2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -693,7 +708,7 @@
         <v>50</v>
       </c>
       <c r="G4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -710,7 +725,7 @@
         <v>50</v>
       </c>
       <c r="G5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -727,7 +742,7 @@
         <v>50</v>
       </c>
       <c r="G6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -783,7 +798,7 @@
         <v>50</v>
       </c>
       <c r="G10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -794,7 +809,7 @@
         <v>50</v>
       </c>
       <c r="G11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -827,7 +842,7 @@
         <v>50</v>
       </c>
       <c r="G14" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -838,7 +853,7 @@
         <v>50</v>
       </c>
       <c r="G15" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -860,7 +875,7 @@
         <v>50</v>
       </c>
       <c r="G17" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="5:7" x14ac:dyDescent="0.25">
@@ -871,7 +886,7 @@
         <v>50</v>
       </c>
       <c r="G18" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="5:7" x14ac:dyDescent="0.25">
@@ -882,7 +897,7 @@
         <v>50</v>
       </c>
       <c r="G19" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="5:7" x14ac:dyDescent="0.25">
@@ -893,7 +908,7 @@
         <v>50</v>
       </c>
       <c r="G20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="5:7" x14ac:dyDescent="0.25">
@@ -904,7 +919,7 @@
         <v>50</v>
       </c>
       <c r="G21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="5:7" x14ac:dyDescent="0.25">
@@ -915,7 +930,7 @@
         <v>50</v>
       </c>
       <c r="G22" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="5:7" x14ac:dyDescent="0.25">
@@ -926,7 +941,7 @@
         <v>50</v>
       </c>
       <c r="G23" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="5:7" x14ac:dyDescent="0.25">
@@ -981,7 +996,7 @@
         <v>50</v>
       </c>
       <c r="G28" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="5:7" x14ac:dyDescent="0.25">
@@ -992,7 +1007,7 @@
         <v>50</v>
       </c>
       <c r="G29" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="5:7" x14ac:dyDescent="0.25">
@@ -1003,7 +1018,7 @@
         <v>50</v>
       </c>
       <c r="G30" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="5:7" x14ac:dyDescent="0.25">
@@ -1014,7 +1029,7 @@
         <v>50</v>
       </c>
       <c r="G31" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="5:7" x14ac:dyDescent="0.25">
@@ -1025,7 +1040,7 @@
         <v>50</v>
       </c>
       <c r="G32" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="5:7" x14ac:dyDescent="0.25">
@@ -1036,7 +1051,7 @@
         <v>50</v>
       </c>
       <c r="G33" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="5:7" x14ac:dyDescent="0.25">
@@ -1047,7 +1062,7 @@
         <v>50</v>
       </c>
       <c r="G34" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="5:7" x14ac:dyDescent="0.25">
@@ -1058,7 +1073,7 @@
         <v>50</v>
       </c>
       <c r="G35" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="5:7" x14ac:dyDescent="0.25">
@@ -1069,7 +1084,7 @@
         <v>50</v>
       </c>
       <c r="G36" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37" spans="5:7" x14ac:dyDescent="0.25">
@@ -1080,7 +1095,7 @@
         <v>50</v>
       </c>
       <c r="G37" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="5:7" x14ac:dyDescent="0.25">
@@ -1091,7 +1106,7 @@
         <v>50</v>
       </c>
       <c r="G38" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39" spans="5:7" x14ac:dyDescent="0.25">
@@ -1102,7 +1117,7 @@
         <v>50</v>
       </c>
       <c r="G39" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="5:7" x14ac:dyDescent="0.25">
@@ -1146,7 +1161,7 @@
         <v>50</v>
       </c>
       <c r="G43" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="5:7" x14ac:dyDescent="0.25">
@@ -1157,6 +1172,39 @@
         <v>50</v>
       </c>
       <c r="G44" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="45" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E45" t="s">
+        <v>61</v>
+      </c>
+      <c r="F45" t="s">
+        <v>62</v>
+      </c>
+      <c r="G45" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="46" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E46" t="s">
+        <v>63</v>
+      </c>
+      <c r="F46" t="s">
+        <v>50</v>
+      </c>
+      <c r="G46" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="47" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E47" t="s">
+        <v>64</v>
+      </c>
+      <c r="F47" t="s">
+        <v>50</v>
+      </c>
+      <c r="G47" t="s">
         <v>51</v>
       </c>
     </row>

</xml_diff>

<commit_message>
third round, almost done still a few discrapancies and cant finish all due to computational restraint
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\broos.nafthali\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C114B4-C98E-42FE-AF05-F2DF5806318D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF9BD25E-BB33-4648-81C4-854AC6ECCAFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -759,7 +759,7 @@
         <v>50</v>
       </c>
       <c r="G7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -776,7 +776,7 @@
         <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -787,7 +787,7 @@
         <v>50</v>
       </c>
       <c r="G9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -1128,7 +1128,7 @@
         <v>50</v>
       </c>
       <c r="G40" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="41" spans="5:7" x14ac:dyDescent="0.25">
@@ -1139,7 +1139,7 @@
         <v>50</v>
       </c>
       <c r="G41" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="5:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
third round, with some altercations
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\broos.nafthali\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\bz.ad.minbuza.local\Data\users\broos.nafthali\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF9BD25E-BB33-4648-81C4-854AC6ECCAFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC77FDBF-9979-43C4-A399-AB2CCA49BB53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -750,7 +750,7 @@
         <v>58</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s">
         <v>12</v>
@@ -767,7 +767,7 @@
         <v>59</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
         <v>13</v>
@@ -952,7 +952,7 @@
         <v>50</v>
       </c>
       <c r="G24" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="5:7" x14ac:dyDescent="0.25">
@@ -963,7 +963,7 @@
         <v>50</v>
       </c>
       <c r="G25" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="5:7" x14ac:dyDescent="0.25">
@@ -974,7 +974,7 @@
         <v>50</v>
       </c>
       <c r="G26" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="5:7" x14ac:dyDescent="0.25">
@@ -985,7 +985,7 @@
         <v>50</v>
       </c>
       <c r="G27" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="5:7" x14ac:dyDescent="0.25">
@@ -996,7 +996,7 @@
         <v>50</v>
       </c>
       <c r="G28" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="5:7" x14ac:dyDescent="0.25">

</xml_diff>